<commit_message>
feat: VMU1 site pack uses booking N0 and field-like iron frames
Wire site-only estimate to pack_effective booking; model FST crates as 1.1/2/4m mix from loading lists so autonomous N0 lands at 2 instead of 15 solid-outer cabinets.
</commit_message>
<xml_diff>
--- a/output/vmu1_site_only/materials_vmu1_site_remaining.xlsx
+++ b/output/vmu1_site_only/materials_vmu1_site_remaining.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L157"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#1</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#1</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4598,19 +4598,19 @@
         <v>1</v>
       </c>
       <c r="E84" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F84" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G84" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H84" t="n">
         <v>1100</v>
       </c>
       <c r="I84" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=1/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=1/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#2</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#2</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4648,19 +4648,19 @@
         <v>1</v>
       </c>
       <c r="E85" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F85" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G85" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H85" t="n">
         <v>1100</v>
       </c>
       <c r="I85" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=2/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=2/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#3</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#3</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4698,19 +4698,19 @@
         <v>1</v>
       </c>
       <c r="E86" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F86" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G86" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H86" t="n">
         <v>1100</v>
       </c>
       <c r="I86" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
@@ -4719,7 +4719,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=3/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=3/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -4736,7 +4736,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#4</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#4</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4748,19 +4748,19 @@
         <v>1</v>
       </c>
       <c r="E87" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F87" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G87" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H87" t="n">
         <v>1100</v>
       </c>
       <c r="I87" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -4769,7 +4769,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=4/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=4/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -4786,7 +4786,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#5</t>
+          <t>2米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#5</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4798,19 +4798,19 @@
         <v>1</v>
       </c>
       <c r="E88" t="n">
-        <v>450</v>
+        <v>1340</v>
       </c>
       <c r="F88" t="n">
-        <v>450</v>
+        <v>1340</v>
       </c>
       <c r="G88" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="H88" t="n">
         <v>1100</v>
       </c>
       <c r="I88" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
@@ -4819,7 +4819,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=5/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=5/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -4836,7 +4836,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#6</t>
+          <t>4米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#6</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -4848,10 +4848,10 @@
         <v>1</v>
       </c>
       <c r="E89" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="F89" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G89" t="n">
         <v>4000</v>
@@ -4860,7 +4860,7 @@
         <v>1100</v>
       </c>
       <c r="I89" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
@@ -4869,7 +4869,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=6/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=6/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#7</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#7</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4898,19 +4898,19 @@
         <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F90" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G90" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H90" t="n">
         <v>1100</v>
       </c>
       <c r="I90" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=7/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=7/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#8</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#8</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4948,19 +4948,19 @@
         <v>1</v>
       </c>
       <c r="E91" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F91" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G91" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H91" t="n">
         <v>1100</v>
       </c>
       <c r="I91" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
@@ -4969,7 +4969,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=8/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=8/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#9</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#9</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4998,19 +4998,19 @@
         <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F92" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G92" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H92" t="n">
         <v>1100</v>
       </c>
       <c r="I92" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J92" t="inlineStr">
         <is>
@@ -5019,7 +5019,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=9/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=9/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#10</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#10</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -5048,19 +5048,19 @@
         <v>1</v>
       </c>
       <c r="E93" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F93" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G93" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H93" t="n">
         <v>1100</v>
       </c>
       <c r="I93" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
@@ -5069,7 +5069,7 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=10/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=10/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#11</t>
+          <t>2米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#11</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -5098,19 +5098,19 @@
         <v>1</v>
       </c>
       <c r="E94" t="n">
-        <v>450</v>
+        <v>1340</v>
       </c>
       <c r="F94" t="n">
-        <v>450</v>
+        <v>1340</v>
       </c>
       <c r="G94" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="H94" t="n">
         <v>1100</v>
       </c>
       <c r="I94" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J94" t="inlineStr">
         <is>
@@ -5119,7 +5119,7 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=11/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=11/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#12</t>
+          <t>4米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#12</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -5148,10 +5148,10 @@
         <v>1</v>
       </c>
       <c r="E95" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="F95" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G95" t="n">
         <v>4000</v>
@@ -5160,7 +5160,7 @@
         <v>1100</v>
       </c>
       <c r="I95" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=12/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=12/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#13</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#13</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -5198,19 +5198,19 @@
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F96" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G96" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H96" t="n">
         <v>1100</v>
       </c>
       <c r="I96" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -5219,7 +5219,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=13/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=13/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -5236,7 +5236,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#14</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#14</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -5248,19 +5248,19 @@
         <v>1</v>
       </c>
       <c r="E97" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F97" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G97" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H97" t="n">
         <v>1100</v>
       </c>
       <c r="I97" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=14/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=14/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -5286,7 +5286,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#15</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#15</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -5298,19 +5298,19 @@
         <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F98" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G98" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H98" t="n">
         <v>1100</v>
       </c>
       <c r="I98" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
@@ -5319,7 +5319,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=15/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=15/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -5336,7 +5336,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#16</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#16</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -5348,19 +5348,19 @@
         <v>1</v>
       </c>
       <c r="E99" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F99" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G99" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H99" t="n">
         <v>1100</v>
       </c>
       <c r="I99" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J99" t="inlineStr">
         <is>
@@ -5369,7 +5369,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=16/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=16/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -5386,7 +5386,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#17</t>
+          <t>2米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#17</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -5398,19 +5398,19 @@
         <v>1</v>
       </c>
       <c r="E100" t="n">
-        <v>450</v>
+        <v>1340</v>
       </c>
       <c r="F100" t="n">
-        <v>450</v>
+        <v>1340</v>
       </c>
       <c r="G100" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="H100" t="n">
         <v>1100</v>
       </c>
       <c r="I100" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
@@ -5419,7 +5419,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=17/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=17/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -5436,7 +5436,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#18</t>
+          <t>4米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#18</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -5448,10 +5448,10 @@
         <v>1</v>
       </c>
       <c r="E101" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="F101" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G101" t="n">
         <v>4000</v>
@@ -5460,7 +5460,7 @@
         <v>1100</v>
       </c>
       <c r="I101" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
@@ -5469,7 +5469,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=18/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=18/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">
@@ -5486,7 +5486,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#19</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#19</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -5498,19 +5498,19 @@
         <v>1</v>
       </c>
       <c r="E102" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F102" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G102" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H102" t="n">
         <v>1100</v>
       </c>
       <c r="I102" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
@@ -5519,7 +5519,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=19/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=19/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#20</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#20</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -5548,19 +5548,19 @@
         <v>1</v>
       </c>
       <c r="E103" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F103" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G103" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H103" t="n">
         <v>1100</v>
       </c>
       <c r="I103" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J103" t="inlineStr">
         <is>
@@ -5569,7 +5569,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=20/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=20/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#21</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#21</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -5598,19 +5598,19 @@
         <v>1</v>
       </c>
       <c r="E104" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F104" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G104" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H104" t="n">
         <v>1100</v>
       </c>
       <c r="I104" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
@@ -5619,7 +5619,7 @@
       </c>
       <c r="K104" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=21/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=21/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L104" t="inlineStr">
@@ -5636,7 +5636,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#22</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#22</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -5648,19 +5648,19 @@
         <v>1</v>
       </c>
       <c r="E105" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F105" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G105" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H105" t="n">
         <v>1100</v>
       </c>
       <c r="I105" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
@@ -5669,7 +5669,7 @@
       </c>
       <c r="K105" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=22/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=22/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L105" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#23</t>
+          <t>2米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#23</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -5698,19 +5698,19 @@
         <v>1</v>
       </c>
       <c r="E106" t="n">
-        <v>450</v>
+        <v>1340</v>
       </c>
       <c r="F106" t="n">
-        <v>450</v>
+        <v>1340</v>
       </c>
       <c r="G106" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="H106" t="n">
         <v>1100</v>
       </c>
       <c r="I106" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J106" t="inlineStr">
         <is>
@@ -5719,7 +5719,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=23/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=23/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#24</t>
+          <t>4米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#24</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -5748,10 +5748,10 @@
         <v>1</v>
       </c>
       <c r="E107" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="F107" t="n">
-        <v>450</v>
+        <v>1450</v>
       </c>
       <c r="G107" t="n">
         <v>4000</v>
@@ -5760,7 +5760,7 @@
         <v>1100</v>
       </c>
       <c r="I107" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J107" t="inlineStr">
         <is>
@@ -5769,7 +5769,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=24/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=24/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#25</t>
+          <t>1.1米铁件架×80件/架 raw=1998 | SLTO-VMU-0001-FST0003#25</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -5798,19 +5798,19 @@
         <v>1</v>
       </c>
       <c r="E108" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="F108" t="n">
-        <v>450</v>
+        <v>1280</v>
       </c>
       <c r="G108" t="n">
-        <v>4000</v>
+        <v>1100</v>
       </c>
       <c r="H108" t="n">
         <v>1100</v>
       </c>
       <c r="I108" t="n">
-        <v>1200</v>
+        <v>1750</v>
       </c>
       <c r="J108" t="inlineStr">
         <is>
@@ -5819,7 +5819,7 @@
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=25/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=1998.0; crate=25/25; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
@@ -5836,7 +5836,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#26</t>
+          <t>吊具 | SLTO-VMU-0001-FST0017#1</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -5848,28 +5848,28 @@
         <v>1</v>
       </c>
       <c r="E109" t="n">
-        <v>450</v>
+        <v>45</v>
       </c>
       <c r="F109" t="n">
-        <v>450</v>
+        <v>45</v>
       </c>
       <c r="G109" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="H109" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="I109" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>SLTO-VMU-0001-FST0003</t>
+          <t>SLTO-VMU-0001-FST0017</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=26/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=4.0; crate=1/4; arr=0.0; pend=4.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L109" t="inlineStr">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#27</t>
+          <t>吊具 | SLTO-VMU-0001-FST0017#2</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -5898,28 +5898,28 @@
         <v>1</v>
       </c>
       <c r="E110" t="n">
-        <v>450</v>
+        <v>45</v>
       </c>
       <c r="F110" t="n">
-        <v>450</v>
+        <v>45</v>
       </c>
       <c r="G110" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="H110" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="I110" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>SLTO-VMU-0001-FST0003</t>
+          <t>SLTO-VMU-0001-FST0017</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=27/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=4.0; crate=2/4; arr=0.0; pend=4.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L110" t="inlineStr">
@@ -5936,7 +5936,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#28</t>
+          <t>吊具 | SLTO-VMU-0001-FST0017#3</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -5948,28 +5948,28 @@
         <v>1</v>
       </c>
       <c r="E111" t="n">
-        <v>450</v>
+        <v>45</v>
       </c>
       <c r="F111" t="n">
-        <v>450</v>
+        <v>45</v>
       </c>
       <c r="G111" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="H111" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="I111" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>SLTO-VMU-0001-FST0003</t>
+          <t>SLTO-VMU-0001-FST0017</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=28/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=4.0; crate=3/4; arr=0.0; pend=4.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L111" t="inlineStr">
@@ -5986,7 +5986,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#29</t>
+          <t>吊具 | SLTO-VMU-0001-FST0017#4</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -5998,28 +5998,28 @@
         <v>1</v>
       </c>
       <c r="E112" t="n">
-        <v>450</v>
+        <v>45</v>
       </c>
       <c r="F112" t="n">
-        <v>450</v>
+        <v>45</v>
       </c>
       <c r="G112" t="n">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="H112" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="I112" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>SLTO-VMU-0001-FST0003</t>
+          <t>SLTO-VMU-0001-FST0017</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=29/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=4.0; crate=4/4; arr=0.0; pend=4.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L112" t="inlineStr">
@@ -6036,7 +6036,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#30</t>
+          <t>钢垫片箱×60/箱 | SLTO-VMU-0001-FST0022#1</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -6048,28 +6048,28 @@
         <v>1</v>
       </c>
       <c r="E113" t="n">
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="F113" t="n">
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="G113" t="n">
-        <v>4000</v>
+        <v>1200</v>
       </c>
       <c r="H113" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="I113" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>SLTO-VMU-0001-FST0003</t>
+          <t>SLTO-VMU-0001-FST0022</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=30/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=189.0; crate=1/3; arr=0.0; pend=189.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L113" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#31</t>
+          <t>钢垫片箱×60/箱 | SLTO-VMU-0001-FST0022#2</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -6098,28 +6098,28 @@
         <v>1</v>
       </c>
       <c r="E114" t="n">
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="F114" t="n">
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="G114" t="n">
-        <v>4000</v>
+        <v>1200</v>
       </c>
       <c r="H114" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="I114" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>SLTO-VMU-0001-FST0003</t>
+          <t>SLTO-VMU-0001-FST0022</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=31/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=189.0; crate=2/3; arr=0.0; pend=189.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L114" t="inlineStr">
@@ -6136,7 +6136,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#32</t>
+          <t>钢垫片箱×60/箱 | SLTO-VMU-0001-FST0022#3</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -6148,2131 +6148,31 @@
         <v>1</v>
       </c>
       <c r="E115" t="n">
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="F115" t="n">
-        <v>450</v>
+        <v>150</v>
       </c>
       <c r="G115" t="n">
-        <v>4000</v>
+        <v>1200</v>
       </c>
       <c r="H115" t="n">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="I115" t="n">
-        <v>1200</v>
+        <v>600</v>
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>SLTO-VMU-0001-FST0003</t>
+          <t>SLTO-VMU-0001-FST0022</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>dest=工地; raw_qty=1998.0; crate=32/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
+          <t>dest=工地; raw_qty=189.0; crate=3/3; arr=0.0; pend=189.0; dims=crate_equiv_est</t>
         </is>
       </c>
       <c r="L115" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>S115</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#33</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D116" t="n">
-        <v>1</v>
-      </c>
-      <c r="E116" t="n">
-        <v>450</v>
-      </c>
-      <c r="F116" t="n">
-        <v>450</v>
-      </c>
-      <c r="G116" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H116" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I116" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J116" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K116" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=33/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L116" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>S116</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#34</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D117" t="n">
-        <v>1</v>
-      </c>
-      <c r="E117" t="n">
-        <v>450</v>
-      </c>
-      <c r="F117" t="n">
-        <v>450</v>
-      </c>
-      <c r="G117" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H117" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I117" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J117" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K117" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=34/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L117" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>S117</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#35</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D118" t="n">
-        <v>1</v>
-      </c>
-      <c r="E118" t="n">
-        <v>450</v>
-      </c>
-      <c r="F118" t="n">
-        <v>450</v>
-      </c>
-      <c r="G118" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H118" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I118" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J118" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K118" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=35/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L118" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>S118</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#36</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D119" t="n">
-        <v>1</v>
-      </c>
-      <c r="E119" t="n">
-        <v>450</v>
-      </c>
-      <c r="F119" t="n">
-        <v>450</v>
-      </c>
-      <c r="G119" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H119" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I119" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J119" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=36/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L119" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>S119</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#37</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D120" t="n">
-        <v>1</v>
-      </c>
-      <c r="E120" t="n">
-        <v>450</v>
-      </c>
-      <c r="F120" t="n">
-        <v>450</v>
-      </c>
-      <c r="G120" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H120" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I120" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J120" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=37/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L120" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>S120</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#38</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D121" t="n">
-        <v>1</v>
-      </c>
-      <c r="E121" t="n">
-        <v>450</v>
-      </c>
-      <c r="F121" t="n">
-        <v>450</v>
-      </c>
-      <c r="G121" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H121" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I121" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J121" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K121" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=38/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L121" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>S121</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#39</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D122" t="n">
-        <v>1</v>
-      </c>
-      <c r="E122" t="n">
-        <v>450</v>
-      </c>
-      <c r="F122" t="n">
-        <v>450</v>
-      </c>
-      <c r="G122" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H122" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I122" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J122" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=39/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L122" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>S122</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#40</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D123" t="n">
-        <v>1</v>
-      </c>
-      <c r="E123" t="n">
-        <v>450</v>
-      </c>
-      <c r="F123" t="n">
-        <v>450</v>
-      </c>
-      <c r="G123" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H123" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I123" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J123" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=40/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L123" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>S123</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#41</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E124" t="n">
-        <v>450</v>
-      </c>
-      <c r="F124" t="n">
-        <v>450</v>
-      </c>
-      <c r="G124" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H124" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I124" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=41/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L124" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>S124</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#42</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D125" t="n">
-        <v>1</v>
-      </c>
-      <c r="E125" t="n">
-        <v>450</v>
-      </c>
-      <c r="F125" t="n">
-        <v>450</v>
-      </c>
-      <c r="G125" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H125" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I125" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J125" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=42/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>S125</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#43</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E126" t="n">
-        <v>450</v>
-      </c>
-      <c r="F126" t="n">
-        <v>450</v>
-      </c>
-      <c r="G126" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H126" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I126" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J126" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=43/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L126" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>S126</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#44</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D127" t="n">
-        <v>1</v>
-      </c>
-      <c r="E127" t="n">
-        <v>450</v>
-      </c>
-      <c r="F127" t="n">
-        <v>450</v>
-      </c>
-      <c r="G127" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H127" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I127" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J127" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=44/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L127" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>S127</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#45</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D128" t="n">
-        <v>1</v>
-      </c>
-      <c r="E128" t="n">
-        <v>450</v>
-      </c>
-      <c r="F128" t="n">
-        <v>450</v>
-      </c>
-      <c r="G128" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H128" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I128" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J128" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K128" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=45/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L128" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>S128</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#46</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D129" t="n">
-        <v>1</v>
-      </c>
-      <c r="E129" t="n">
-        <v>450</v>
-      </c>
-      <c r="F129" t="n">
-        <v>450</v>
-      </c>
-      <c r="G129" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H129" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I129" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J129" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=46/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L129" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>S129</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#47</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D130" t="n">
-        <v>1</v>
-      </c>
-      <c r="E130" t="n">
-        <v>450</v>
-      </c>
-      <c r="F130" t="n">
-        <v>450</v>
-      </c>
-      <c r="G130" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H130" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I130" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J130" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K130" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=47/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L130" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>S130</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#48</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D131" t="n">
-        <v>1</v>
-      </c>
-      <c r="E131" t="n">
-        <v>450</v>
-      </c>
-      <c r="F131" t="n">
-        <v>450</v>
-      </c>
-      <c r="G131" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H131" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I131" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J131" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K131" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=48/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L131" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>S131</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#49</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D132" t="n">
-        <v>1</v>
-      </c>
-      <c r="E132" t="n">
-        <v>450</v>
-      </c>
-      <c r="F132" t="n">
-        <v>450</v>
-      </c>
-      <c r="G132" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H132" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I132" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J132" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K132" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=49/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L132" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>S132</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#50</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D133" t="n">
-        <v>1</v>
-      </c>
-      <c r="E133" t="n">
-        <v>450</v>
-      </c>
-      <c r="F133" t="n">
-        <v>450</v>
-      </c>
-      <c r="G133" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H133" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I133" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J133" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K133" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=50/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L133" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>S133</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#51</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D134" t="n">
-        <v>1</v>
-      </c>
-      <c r="E134" t="n">
-        <v>450</v>
-      </c>
-      <c r="F134" t="n">
-        <v>450</v>
-      </c>
-      <c r="G134" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H134" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I134" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J134" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K134" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=51/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L134" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>S134</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#52</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D135" t="n">
-        <v>1</v>
-      </c>
-      <c r="E135" t="n">
-        <v>450</v>
-      </c>
-      <c r="F135" t="n">
-        <v>450</v>
-      </c>
-      <c r="G135" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H135" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I135" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J135" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K135" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=52/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L135" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>S135</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#53</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D136" t="n">
-        <v>1</v>
-      </c>
-      <c r="E136" t="n">
-        <v>450</v>
-      </c>
-      <c r="F136" t="n">
-        <v>450</v>
-      </c>
-      <c r="G136" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H136" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I136" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J136" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K136" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=53/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L136" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>S136</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#54</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D137" t="n">
-        <v>1</v>
-      </c>
-      <c r="E137" t="n">
-        <v>450</v>
-      </c>
-      <c r="F137" t="n">
-        <v>450</v>
-      </c>
-      <c r="G137" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H137" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I137" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K137" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=54/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L137" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>S137</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#55</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D138" t="n">
-        <v>1</v>
-      </c>
-      <c r="E138" t="n">
-        <v>450</v>
-      </c>
-      <c r="F138" t="n">
-        <v>450</v>
-      </c>
-      <c r="G138" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H138" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I138" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J138" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K138" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=55/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L138" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>S138</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#56</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D139" t="n">
-        <v>1</v>
-      </c>
-      <c r="E139" t="n">
-        <v>450</v>
-      </c>
-      <c r="F139" t="n">
-        <v>450</v>
-      </c>
-      <c r="G139" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H139" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I139" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J139" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K139" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=56/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L139" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>S139</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#57</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D140" t="n">
-        <v>1</v>
-      </c>
-      <c r="E140" t="n">
-        <v>450</v>
-      </c>
-      <c r="F140" t="n">
-        <v>450</v>
-      </c>
-      <c r="G140" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H140" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I140" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J140" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K140" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=57/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L140" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>S140</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#58</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D141" t="n">
-        <v>1</v>
-      </c>
-      <c r="E141" t="n">
-        <v>450</v>
-      </c>
-      <c r="F141" t="n">
-        <v>450</v>
-      </c>
-      <c r="G141" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H141" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I141" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J141" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K141" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=58/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L141" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>S141</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#59</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D142" t="n">
-        <v>1</v>
-      </c>
-      <c r="E142" t="n">
-        <v>450</v>
-      </c>
-      <c r="F142" t="n">
-        <v>450</v>
-      </c>
-      <c r="G142" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H142" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I142" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J142" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K142" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=59/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L142" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>S142</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#60</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D143" t="n">
-        <v>1</v>
-      </c>
-      <c r="E143" t="n">
-        <v>450</v>
-      </c>
-      <c r="F143" t="n">
-        <v>450</v>
-      </c>
-      <c r="G143" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H143" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I143" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J143" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K143" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=60/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L143" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>S143</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#61</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D144" t="n">
-        <v>1</v>
-      </c>
-      <c r="E144" t="n">
-        <v>450</v>
-      </c>
-      <c r="F144" t="n">
-        <v>450</v>
-      </c>
-      <c r="G144" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H144" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I144" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J144" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K144" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=61/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L144" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>S144</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#62</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D145" t="n">
-        <v>1</v>
-      </c>
-      <c r="E145" t="n">
-        <v>450</v>
-      </c>
-      <c r="F145" t="n">
-        <v>450</v>
-      </c>
-      <c r="G145" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H145" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I145" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J145" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K145" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=62/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L145" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>S145</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#63</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D146" t="n">
-        <v>1</v>
-      </c>
-      <c r="E146" t="n">
-        <v>450</v>
-      </c>
-      <c r="F146" t="n">
-        <v>450</v>
-      </c>
-      <c r="G146" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H146" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I146" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J146" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=63/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L146" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>S146</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#64</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D147" t="n">
-        <v>1</v>
-      </c>
-      <c r="E147" t="n">
-        <v>450</v>
-      </c>
-      <c r="F147" t="n">
-        <v>450</v>
-      </c>
-      <c r="G147" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H147" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I147" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J147" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K147" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=64/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L147" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>S147</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#65</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D148" t="n">
-        <v>1</v>
-      </c>
-      <c r="E148" t="n">
-        <v>450</v>
-      </c>
-      <c r="F148" t="n">
-        <v>450</v>
-      </c>
-      <c r="G148" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H148" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I148" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J148" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K148" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=65/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L148" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>S148</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#66</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D149" t="n">
-        <v>1</v>
-      </c>
-      <c r="E149" t="n">
-        <v>450</v>
-      </c>
-      <c r="F149" t="n">
-        <v>450</v>
-      </c>
-      <c r="G149" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H149" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I149" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J149" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K149" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=66/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L149" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>S149</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>铁件架×30件/架 raw=1998 | SLTO-VMU-0001-FST0003#67</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D150" t="n">
-        <v>1</v>
-      </c>
-      <c r="E150" t="n">
-        <v>450</v>
-      </c>
-      <c r="F150" t="n">
-        <v>450</v>
-      </c>
-      <c r="G150" t="n">
-        <v>4000</v>
-      </c>
-      <c r="H150" t="n">
-        <v>1100</v>
-      </c>
-      <c r="I150" t="n">
-        <v>1200</v>
-      </c>
-      <c r="J150" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0003</t>
-        </is>
-      </c>
-      <c r="K150" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=1998.0; crate=67/67; arr=0.0; pend=1998.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L150" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>S150</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>吊具 | SLTO-VMU-0001-FST0017#1</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D151" t="n">
-        <v>1</v>
-      </c>
-      <c r="E151" t="n">
-        <v>45</v>
-      </c>
-      <c r="F151" t="n">
-        <v>45</v>
-      </c>
-      <c r="G151" t="n">
-        <v>2000</v>
-      </c>
-      <c r="H151" t="n">
-        <v>800</v>
-      </c>
-      <c r="I151" t="n">
-        <v>600</v>
-      </c>
-      <c r="J151" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0017</t>
-        </is>
-      </c>
-      <c r="K151" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=4.0; crate=1/4; arr=0.0; pend=4.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L151" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>S151</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>吊具 | SLTO-VMU-0001-FST0017#2</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D152" t="n">
-        <v>1</v>
-      </c>
-      <c r="E152" t="n">
-        <v>45</v>
-      </c>
-      <c r="F152" t="n">
-        <v>45</v>
-      </c>
-      <c r="G152" t="n">
-        <v>2000</v>
-      </c>
-      <c r="H152" t="n">
-        <v>800</v>
-      </c>
-      <c r="I152" t="n">
-        <v>600</v>
-      </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0017</t>
-        </is>
-      </c>
-      <c r="K152" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=4.0; crate=2/4; arr=0.0; pend=4.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L152" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>S152</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>吊具 | SLTO-VMU-0001-FST0017#3</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D153" t="n">
-        <v>1</v>
-      </c>
-      <c r="E153" t="n">
-        <v>45</v>
-      </c>
-      <c r="F153" t="n">
-        <v>45</v>
-      </c>
-      <c r="G153" t="n">
-        <v>2000</v>
-      </c>
-      <c r="H153" t="n">
-        <v>800</v>
-      </c>
-      <c r="I153" t="n">
-        <v>600</v>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0017</t>
-        </is>
-      </c>
-      <c r="K153" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=4.0; crate=3/4; arr=0.0; pend=4.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L153" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>S153</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>吊具 | SLTO-VMU-0001-FST0017#4</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D154" t="n">
-        <v>1</v>
-      </c>
-      <c r="E154" t="n">
-        <v>45</v>
-      </c>
-      <c r="F154" t="n">
-        <v>45</v>
-      </c>
-      <c r="G154" t="n">
-        <v>2000</v>
-      </c>
-      <c r="H154" t="n">
-        <v>800</v>
-      </c>
-      <c r="I154" t="n">
-        <v>600</v>
-      </c>
-      <c r="J154" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0017</t>
-        </is>
-      </c>
-      <c r="K154" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=4.0; crate=4/4; arr=0.0; pend=4.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L154" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>S154</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>钢垫片箱×60/箱 | SLTO-VMU-0001-FST0022#1</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D155" t="n">
-        <v>1</v>
-      </c>
-      <c r="E155" t="n">
-        <v>150</v>
-      </c>
-      <c r="F155" t="n">
-        <v>150</v>
-      </c>
-      <c r="G155" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H155" t="n">
-        <v>800</v>
-      </c>
-      <c r="I155" t="n">
-        <v>600</v>
-      </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0022</t>
-        </is>
-      </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=189.0; crate=1/3; arr=0.0; pend=189.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L155" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>S155</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>钢垫片箱×60/箱 | SLTO-VMU-0001-FST0022#2</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D156" t="n">
-        <v>1</v>
-      </c>
-      <c r="E156" t="n">
-        <v>150</v>
-      </c>
-      <c r="F156" t="n">
-        <v>150</v>
-      </c>
-      <c r="G156" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H156" t="n">
-        <v>800</v>
-      </c>
-      <c r="I156" t="n">
-        <v>600</v>
-      </c>
-      <c r="J156" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0022</t>
-        </is>
-      </c>
-      <c r="K156" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=189.0; crate=2/3; arr=0.0; pend=189.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L156" t="inlineStr">
-        <is>
-          <t>工地</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>S156</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>钢垫片箱×60/箱 | SLTO-VMU-0001-FST0022#3</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>13—铁件</t>
-        </is>
-      </c>
-      <c r="D157" t="n">
-        <v>1</v>
-      </c>
-      <c r="E157" t="n">
-        <v>150</v>
-      </c>
-      <c r="F157" t="n">
-        <v>150</v>
-      </c>
-      <c r="G157" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H157" t="n">
-        <v>800</v>
-      </c>
-      <c r="I157" t="n">
-        <v>600</v>
-      </c>
-      <c r="J157" t="inlineStr">
-        <is>
-          <t>SLTO-VMU-0001-FST0022</t>
-        </is>
-      </c>
-      <c r="K157" t="inlineStr">
-        <is>
-          <t>dest=工地; raw_qty=189.0; crate=3/3; arr=0.0; pend=189.0; dims=crate_equiv_est</t>
-        </is>
-      </c>
-      <c r="L157" t="inlineStr">
         <is>
           <t>工地</t>
         </is>

</xml_diff>